<commit_message>
Add full Dotan platform: tasks calendar, commander walls, users wall, attendance, birthdays, messages
- Add Task, CommanderPost models and migrations
- Import 337 tasks from ICS calendar file
- Build tasks page with week/list views, alerts, and filtering
- Build commander wall with dedicated pages per leader (8 commanders set)
- Build users wall with search, team filtering, and detail modals
- Build attendance (מצל) page with team stats
- Build birthdays wall with monthly calendar view
- Build message board with create/delete/pin
- Add session persistence (30 days)
- Add "Made by עידן סימנטוב צוות 16" footer
- Fix 12 user name mismatches from xlsx
- Mobile-responsive design throughout
- Updated login xlsx with all 60 users

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/users-login-list.xlsx
+++ b/users-login-list.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="משתמשים" sheetId="1" r:id="rId1"/>
+    <sheet name="נתוני התחברות" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,12 +397,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:G61"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="3" max="3" width="28.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -410,858 +413,1395 @@
         <v>שם</v>
       </c>
       <c r="B1" t="str">
+        <v>אימייל (שם משתמש)</v>
+      </c>
+      <c r="C1" t="str">
+        <v>סיסמה</v>
+      </c>
+      <c r="D1" t="str">
+        <v>צוות</v>
+      </c>
+      <c r="E1" t="str">
         <v>חדר</v>
       </c>
-      <c r="C1" t="str">
-        <v>אימייל</v>
-      </c>
-      <c r="D1" t="str">
-        <v>סיסמה</v>
+      <c r="F1" t="str">
+        <v>טלפון</v>
+      </c>
+      <c r="G1" t="str">
+        <v>תפקיד</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>רועי דדון</v>
+        <v>אייל מוזר</v>
       </c>
       <c r="B2" t="str">
-        <v>219</v>
+        <v>user.217.24@laundry.app</v>
       </c>
       <c r="C2" t="str">
-        <v>user.219.1@laundry.app</v>
-      </c>
-      <c r="D2" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D2">
+        <v>14</v>
+      </c>
+      <c r="E2" t="str">
+        <v>217</v>
+      </c>
+      <c r="F2" t="str">
+        <v>0523344007</v>
+      </c>
+      <c r="G2" t="str">
+        <v>קב"ט</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>יובל ישר</v>
+        <v>אלה בן גיא</v>
       </c>
       <c r="B3" t="str">
-        <v>219</v>
+        <v>user.401.41@laundry.app</v>
       </c>
       <c r="C3" t="str">
-        <v>user.219.2@laundry.app</v>
-      </c>
-      <c r="D3" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D3">
+        <v>14</v>
+      </c>
+      <c r="E3" t="str">
+        <v>401</v>
+      </c>
+      <c r="F3" t="str">
+        <v>0586448455</v>
+      </c>
+      <c r="G3" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>יהונתן אבוקרט</v>
+        <v>דולב כהן</v>
       </c>
       <c r="B4" t="str">
+        <v>user.219.6@laundry.app</v>
+      </c>
+      <c r="C4" t="str">
+        <v>123456</v>
+      </c>
+      <c r="D4">
+        <v>14</v>
+      </c>
+      <c r="E4" t="str">
         <v>219</v>
       </c>
-      <c r="C4" t="str">
-        <v>user.219.3@laundry.app</v>
-      </c>
-      <c r="D4" t="str">
-        <v>123456</v>
+      <c r="F4" t="str">
+        <v>0542542104</v>
+      </c>
+      <c r="G4" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>עילי בן אברהם</v>
+        <v>יהלי כוכבא</v>
       </c>
       <c r="B5" t="str">
-        <v>219</v>
+        <v>user.401.39@laundry.app</v>
       </c>
       <c r="C5" t="str">
-        <v>user.219.4@laundry.app</v>
-      </c>
-      <c r="D5" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D5">
+        <v>14</v>
+      </c>
+      <c r="E5" t="str">
+        <v>401</v>
+      </c>
+      <c r="G5" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>עילי גולדשטיין</v>
+        <v>יזן כנעאן</v>
       </c>
       <c r="B6" t="str">
-        <v>219</v>
+        <v>user.307.14@laundry.app</v>
       </c>
       <c r="C6" t="str">
-        <v>user.219.5@laundry.app</v>
-      </c>
-      <c r="D6" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D6">
+        <v>14</v>
+      </c>
+      <c r="E6" t="str">
+        <v>307</v>
+      </c>
+      <c r="F6" t="str">
+        <v>0509700593</v>
+      </c>
+      <c r="G6" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>דולב כהן</v>
+        <v>יעל שושן</v>
       </c>
       <c r="B7" t="str">
-        <v>219</v>
+        <v>user.401.40@laundry.app</v>
       </c>
       <c r="C7" t="str">
-        <v>user.219.6@laundry.app</v>
-      </c>
-      <c r="D7" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D7">
+        <v>14</v>
+      </c>
+      <c r="E7" t="str">
+        <v>401</v>
+      </c>
+      <c r="G7" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>טל הנגבי</v>
+        <v>כפיר ברמן</v>
       </c>
       <c r="B8" t="str">
-        <v>403</v>
+        <v>user.305.32@laundry.app</v>
       </c>
       <c r="C8" t="str">
-        <v>user.403.7@laundry.app</v>
-      </c>
-      <c r="D8" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D8">
+        <v>14</v>
+      </c>
+      <c r="E8" t="str">
+        <v>305</v>
+      </c>
+      <c r="F8" t="str">
+        <v>0505815266</v>
+      </c>
+      <c r="G8" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>מאי צימרמן</v>
+        <v>כרמל מורן</v>
       </c>
       <c r="B9" t="str">
-        <v>403</v>
+        <v>user.401.38@laundry.app</v>
       </c>
       <c r="C9" t="str">
-        <v>user.403.8@laundry.app</v>
-      </c>
-      <c r="D9" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D9">
+        <v>14</v>
+      </c>
+      <c r="E9" t="str">
+        <v>401</v>
+      </c>
+      <c r="F9" t="str">
+        <v>0585651818</v>
+      </c>
+      <c r="G9" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>פיונה פונג</v>
+        <v>לייה אלון</v>
       </c>
       <c r="B10" t="str">
-        <v>403</v>
+        <v>user.407.56@laundry.app</v>
       </c>
       <c r="C10" t="str">
-        <v>user.403.9@laundry.app</v>
-      </c>
-      <c r="D10" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D10">
+        <v>14</v>
+      </c>
+      <c r="E10" t="str">
+        <v>407</v>
+      </c>
+      <c r="F10" t="str">
+        <v>0534253534</v>
+      </c>
+      <c r="G10" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>הילה פינצי</v>
+        <v>מאי צימרמן</v>
       </c>
       <c r="B11" t="str">
+        <v>user.403.8@laundry.app</v>
+      </c>
+      <c r="C11" t="str">
+        <v>123456</v>
+      </c>
+      <c r="D11">
+        <v>14</v>
+      </c>
+      <c r="E11" t="str">
         <v>403</v>
       </c>
-      <c r="C11" t="str">
-        <v>user.403.10@laundry.app</v>
-      </c>
-      <c r="D11" t="str">
-        <v>123456</v>
+      <c r="F11" t="str">
+        <v>0544672912</v>
+      </c>
+      <c r="G11" t="str">
+        <v>קהדית פלוגתית</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>מיקה חיים</v>
+        <v>ענבר שלח</v>
       </c>
       <c r="B12" t="str">
-        <v>403</v>
+        <v>user.411.21@laundry.app</v>
       </c>
       <c r="C12" t="str">
-        <v>user.403.11@laundry.app</v>
-      </c>
-      <c r="D12" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D12">
+        <v>14</v>
+      </c>
+      <c r="E12" t="str">
+        <v>411</v>
+      </c>
+      <c r="F12" t="str">
+        <v>0502202857</v>
+      </c>
+      <c r="G12" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>נועה גלמן</v>
+        <v>פיונה פנג</v>
       </c>
       <c r="B13" t="str">
+        <v>user.403.9@laundry.app</v>
+      </c>
+      <c r="C13" t="str">
+        <v>123456</v>
+      </c>
+      <c r="D13">
+        <v>14</v>
+      </c>
+      <c r="E13" t="str">
         <v>403</v>
       </c>
-      <c r="C13" t="str">
-        <v>user.403.12@laundry.app</v>
-      </c>
-      <c r="D13" t="str">
-        <v>123456</v>
+      <c r="F13" t="str">
+        <v>0528601984</v>
+      </c>
+      <c r="G13" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>אופק מזור</v>
+        <v>רוני קרפט</v>
       </c>
       <c r="B14" t="str">
-        <v>307</v>
+        <v>user.405.44@laundry.app</v>
       </c>
       <c r="C14" t="str">
-        <v>user.307.13@laundry.app</v>
-      </c>
-      <c r="D14" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D14">
+        <v>14</v>
+      </c>
+      <c r="E14" t="str">
+        <v>405</v>
+      </c>
+      <c r="F14" t="str">
+        <v>0522282317</v>
+      </c>
+      <c r="G14" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>יזן כנעאן</v>
+        <v>רותם כוכבי</v>
       </c>
       <c r="B15" t="str">
-        <v>307</v>
+        <v>user.413.28@laundry.app</v>
       </c>
       <c r="C15" t="str">
-        <v>user.307.14@laundry.app</v>
-      </c>
-      <c r="D15" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D15">
+        <v>14</v>
+      </c>
+      <c r="E15" t="str">
+        <v>413</v>
+      </c>
+      <c r="F15" t="str">
+        <v>0522736003</v>
+      </c>
+      <c r="G15" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>עדי ולנשטיין</v>
+        <v>רעות ניר</v>
       </c>
       <c r="B16" t="str">
-        <v>307</v>
+        <v>user.409.51@laundry.app</v>
       </c>
       <c r="C16" t="str">
-        <v>user.307.15@laundry.app</v>
-      </c>
-      <c r="D16" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D16">
+        <v>14</v>
+      </c>
+      <c r="E16" t="str">
+        <v>409</v>
+      </c>
+      <c r="F16" t="str">
+        <v>0587886382</v>
+      </c>
+      <c r="G16" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>אלון זלנפרויד</v>
+        <v>אופק מזור</v>
       </c>
       <c r="B17" t="str">
+        <v>user.307.13@laundry.app</v>
+      </c>
+      <c r="C17" t="str">
+        <v>123456</v>
+      </c>
+      <c r="D17">
+        <v>15</v>
+      </c>
+      <c r="E17" t="str">
         <v>307</v>
       </c>
-      <c r="C17" t="str">
-        <v>user.307.16@laundry.app</v>
-      </c>
-      <c r="D17" t="str">
-        <v>123456</v>
+      <c r="F17" t="str">
+        <v>0558819568</v>
+      </c>
+      <c r="G17" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ורווה טופן</v>
+        <v>איתן אונגר</v>
       </c>
       <c r="B18" t="str">
-        <v>411</v>
+        <v>user.305.33@laundry.app</v>
       </c>
       <c r="C18" t="str">
-        <v>user.411.17@laundry.app</v>
-      </c>
-      <c r="D18" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D18">
+        <v>15</v>
+      </c>
+      <c r="E18" t="str">
+        <v>305</v>
+      </c>
+      <c r="F18" t="str">
+        <v>0584704717</v>
+      </c>
+      <c r="G18" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>נועה בלפור</v>
+        <v>דנה פרידמן</v>
       </c>
       <c r="B19" t="str">
-        <v>411</v>
+        <v>user.409.49@laundry.app</v>
       </c>
       <c r="C19" t="str">
-        <v>user.411.18@laundry.app</v>
-      </c>
-      <c r="D19" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D19">
+        <v>15</v>
+      </c>
+      <c r="E19" t="str">
+        <v>409</v>
+      </c>
+      <c r="F19" t="str">
+        <v>0586267598</v>
+      </c>
+      <c r="G19" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>שני זידמן</v>
+        <v>הודיה יעקבי</v>
       </c>
       <c r="B20" t="str">
-        <v>411</v>
+        <v>user.405.46@laundry.app</v>
       </c>
       <c r="C20" t="str">
-        <v>user.411.19@laundry.app</v>
-      </c>
-      <c r="D20" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D20">
+        <v>15</v>
+      </c>
+      <c r="E20" t="str">
+        <v>405</v>
+      </c>
+      <c r="F20" t="str">
+        <v>0543944481</v>
+      </c>
+      <c r="G20" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>רננה ישראלוב</v>
+        <v>הללי בר יוסף</v>
       </c>
       <c r="B21" t="str">
-        <v>411</v>
+        <v>user.401.37@laundry.app</v>
       </c>
       <c r="C21" t="str">
-        <v>user.411.20@laundry.app</v>
-      </c>
-      <c r="D21" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D21">
+        <v>15</v>
+      </c>
+      <c r="E21" t="str">
+        <v>401</v>
+      </c>
+      <c r="F21" t="str">
+        <v>0523360301</v>
+      </c>
+      <c r="G21" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ענבר שלח</v>
+        <v>ורוורה טופן</v>
       </c>
       <c r="B22" t="str">
+        <v>user.411.17@laundry.app</v>
+      </c>
+      <c r="C22" t="str">
+        <v>123456</v>
+      </c>
+      <c r="D22">
+        <v>15</v>
+      </c>
+      <c r="E22" t="str">
         <v>411</v>
       </c>
-      <c r="C22" t="str">
-        <v>user.411.21@laundry.app</v>
-      </c>
-      <c r="D22" t="str">
-        <v>123456</v>
+      <c r="F22" t="str">
+        <v>0539282069</v>
+      </c>
+      <c r="G22" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>מעין מרדכי</v>
+        <v>טליה פרסט</v>
       </c>
       <c r="B23" t="str">
-        <v>411</v>
+        <v>user.407.57@laundry.app</v>
       </c>
       <c r="C23" t="str">
-        <v>user.411.22@laundry.app</v>
-      </c>
-      <c r="D23" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D23">
+        <v>15</v>
+      </c>
+      <c r="E23" t="str">
+        <v>407</v>
+      </c>
+      <c r="G23" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>דור מנשה קיפגן</v>
+        <v>יניב גופמן</v>
       </c>
       <c r="B24" t="str">
+        <v>user.217.26@laundry.app</v>
+      </c>
+      <c r="C24" t="str">
+        <v>123456</v>
+      </c>
+      <c r="D24">
+        <v>15</v>
+      </c>
+      <c r="E24" t="str">
         <v>217</v>
       </c>
-      <c r="C24" t="str">
-        <v>user.217.23@laundry.app</v>
-      </c>
-      <c r="D24" t="str">
-        <v>123456</v>
+      <c r="F24" t="str">
+        <v>0535259538</v>
+      </c>
+      <c r="G24" t="str">
+        <v>קלפ חזק</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>אייל מזור</v>
+        <v>יערה רחוביצקי</v>
       </c>
       <c r="B25" t="str">
-        <v>217</v>
+        <v>user.413.30@laundry.app</v>
       </c>
       <c r="C25" t="str">
-        <v>user.217.24@laundry.app</v>
-      </c>
-      <c r="D25" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D25">
+        <v>15</v>
+      </c>
+      <c r="E25" t="str">
+        <v>413</v>
+      </c>
+      <c r="F25" t="str">
+        <v>0547726335</v>
+      </c>
+      <c r="G25" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>עידן סימנטוב</v>
+        <v>מאי אילארי</v>
       </c>
       <c r="B26" t="str">
-        <v>217</v>
+        <v>user.405.45@laundry.app</v>
       </c>
       <c r="C26" t="str">
-        <v>user.217.25@laundry.app</v>
-      </c>
-      <c r="D26" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D26">
+        <v>15</v>
+      </c>
+      <c r="E26" t="str">
+        <v>405</v>
+      </c>
+      <c r="F26" t="str">
+        <v>0542131528</v>
+      </c>
+      <c r="G26" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>יניב גופמן</v>
+        <v>מיקה חיים</v>
       </c>
       <c r="B27" t="str">
-        <v>217</v>
+        <v>user.403.11@laundry.app</v>
       </c>
       <c r="C27" t="str">
-        <v>user.217.26@laundry.app</v>
-      </c>
-      <c r="D27" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D27">
+        <v>15</v>
+      </c>
+      <c r="E27" t="str">
+        <v>403</v>
+      </c>
+      <c r="F27" t="str">
+        <v>0543263061</v>
+      </c>
+      <c r="G27" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>יהלי לוי</v>
+        <v>נעמה לביא</v>
       </c>
       <c r="B28" t="str">
-        <v>413</v>
+        <v>user.407.58@laundry.app</v>
       </c>
       <c r="C28" t="str">
-        <v>user.413.27@laundry.app</v>
-      </c>
-      <c r="D28" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D28">
+        <v>15</v>
+      </c>
+      <c r="E28" t="str">
+        <v>407</v>
+      </c>
+      <c r="F28" t="str">
+        <v>0549856665</v>
+      </c>
+      <c r="G28" t="str">
+        <v>קא"רית פלוגתית</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>רותם כוכבי</v>
+        <v>עילי בן אברהם</v>
       </c>
       <c r="B29" t="str">
-        <v>413</v>
+        <v>user.219.4@laundry.app</v>
       </c>
       <c r="C29" t="str">
-        <v>user.413.28@laundry.app</v>
-      </c>
-      <c r="D29" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D29">
+        <v>15</v>
+      </c>
+      <c r="E29" t="str">
+        <v>219</v>
+      </c>
+      <c r="F29" t="str">
+        <v>0584814814</v>
+      </c>
+      <c r="G29" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>אלה פלד</v>
+        <v>עמית שושנה</v>
       </c>
       <c r="B30" t="str">
-        <v>413</v>
+        <v>user.405.43@laundry.app</v>
       </c>
       <c r="C30" t="str">
-        <v>user.413.29@laundry.app</v>
-      </c>
-      <c r="D30" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D30">
+        <v>15</v>
+      </c>
+      <c r="E30" t="str">
+        <v>405</v>
+      </c>
+      <c r="G30" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>יערה רחוביצקי</v>
+        <v>שילת נוימן</v>
       </c>
       <c r="B31" t="str">
-        <v>413</v>
+        <v>user.407.59@laundry.app</v>
       </c>
       <c r="C31" t="str">
-        <v>user.413.30@laundry.app</v>
-      </c>
-      <c r="D31" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D31">
+        <v>15</v>
+      </c>
+      <c r="E31" t="str">
+        <v>407</v>
+      </c>
+      <c r="F31" t="str">
+        <v>0584896070</v>
+      </c>
+      <c r="G31" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>עדן בחרוף</v>
+        <v>שיר סויסה</v>
       </c>
       <c r="B32" t="str">
-        <v>413</v>
+        <v>user.401.42@laundry.app</v>
       </c>
       <c r="C32" t="str">
-        <v>user.413.31@laundry.app</v>
-      </c>
-      <c r="D32" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D32">
+        <v>15</v>
+      </c>
+      <c r="E32" t="str">
+        <v>401</v>
+      </c>
+      <c r="F32" t="str">
+        <v>0549063626</v>
+      </c>
+      <c r="G32" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>כפיר ברמן</v>
+        <v>שני זידמן</v>
       </c>
       <c r="B33" t="str">
-        <v>305</v>
+        <v>user.411.19@laundry.app</v>
       </c>
       <c r="C33" t="str">
-        <v>user.305.32@laundry.app</v>
-      </c>
-      <c r="D33" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D33">
+        <v>15</v>
+      </c>
+      <c r="E33" t="str">
+        <v>411</v>
+      </c>
+      <c r="F33" t="str">
+        <v>0543548854</v>
+      </c>
+      <c r="G33" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>איתן אונגר</v>
+        <v>אורי חדד</v>
       </c>
       <c r="B34" t="str">
+        <v>user.305.35@laundry.app</v>
+      </c>
+      <c r="C34" t="str">
+        <v>123456</v>
+      </c>
+      <c r="D34">
+        <v>16</v>
+      </c>
+      <c r="E34" t="str">
         <v>305</v>
       </c>
-      <c r="C34" t="str">
-        <v>user.305.33@laundry.app</v>
-      </c>
-      <c r="D34" t="str">
-        <v>123456</v>
+      <c r="F34" t="str">
+        <v>0545271266</v>
+      </c>
+      <c r="G34" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>עידן טורקיה</v>
+        <v>אלה פלד</v>
       </c>
       <c r="B35" t="str">
-        <v>305</v>
+        <v>user.413.29@laundry.app</v>
       </c>
       <c r="C35" t="str">
-        <v>user.305.34@laundry.app</v>
-      </c>
-      <c r="D35" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D35">
+        <v>16</v>
+      </c>
+      <c r="E35" t="str">
+        <v>413</v>
+      </c>
+      <c r="F35" t="str">
+        <v>0527071407</v>
+      </c>
+      <c r="G35" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>אורי חדד</v>
+        <v>הילה פינצי</v>
       </c>
       <c r="B36" t="str">
-        <v>305</v>
+        <v>user.403.10@laundry.app</v>
       </c>
       <c r="C36" t="str">
-        <v>user.305.35@laundry.app</v>
-      </c>
-      <c r="D36" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D36">
+        <v>16</v>
+      </c>
+      <c r="E36" t="str">
+        <v>403</v>
+      </c>
+      <c r="F36" t="str">
+        <v>0544271331</v>
+      </c>
+      <c r="G36" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>אוהד אבדי</v>
+        <v>יהלי לוי</v>
       </c>
       <c r="B37" t="str">
-        <v>305</v>
+        <v>user.413.27@laundry.app</v>
       </c>
       <c r="C37" t="str">
-        <v>user.305.36@laundry.app</v>
-      </c>
-      <c r="D37" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D37">
+        <v>16</v>
+      </c>
+      <c r="E37" t="str">
+        <v>413</v>
+      </c>
+      <c r="F37" t="str">
+        <v>0503029952</v>
+      </c>
+      <c r="G37" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>הללי בר יוסף</v>
+        <v>מעיין מרדכי</v>
       </c>
       <c r="B38" t="str">
-        <v>401</v>
+        <v>user.411.22@laundry.app</v>
       </c>
       <c r="C38" t="str">
-        <v>user.401.37@laundry.app</v>
-      </c>
-      <c r="D38" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D38">
+        <v>16</v>
+      </c>
+      <c r="E38" t="str">
+        <v>411</v>
+      </c>
+      <c r="F38" t="str">
+        <v>0506358005</v>
+      </c>
+      <c r="G38" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>כרמל מורן</v>
+        <v>נועה בלפור</v>
       </c>
       <c r="B39" t="str">
-        <v>401</v>
+        <v>user.411.18@laundry.app</v>
       </c>
       <c r="C39" t="str">
-        <v>user.401.38@laundry.app</v>
-      </c>
-      <c r="D39" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D39">
+        <v>16</v>
+      </c>
+      <c r="E39" t="str">
+        <v>411</v>
+      </c>
+      <c r="F39" t="str">
+        <v>0559771379</v>
+      </c>
+      <c r="G39" t="str">
+        <v>קאגית פלוגתית</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>יהלי כוכבא</v>
+        <v>נועה גלמן</v>
       </c>
       <c r="B40" t="str">
-        <v>401</v>
+        <v>user.403.12@laundry.app</v>
       </c>
       <c r="C40" t="str">
-        <v>user.401.39@laundry.app</v>
-      </c>
-      <c r="D40" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D40">
+        <v>16</v>
+      </c>
+      <c r="E40" t="str">
+        <v>403</v>
+      </c>
+      <c r="F40" t="str">
+        <v>0587782888</v>
+      </c>
+      <c r="G40" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>יעל שושן</v>
+        <v>נטע וילונסקי</v>
       </c>
       <c r="B41" t="str">
-        <v>401</v>
+        <v>user.409.53@laundry.app</v>
       </c>
       <c r="C41" t="str">
-        <v>user.401.40@laundry.app</v>
-      </c>
-      <c r="D41" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D41">
+        <v>16</v>
+      </c>
+      <c r="E41" t="str">
+        <v>409</v>
+      </c>
+      <c r="F41" t="str">
+        <v>0587002302</v>
+      </c>
+      <c r="G41" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>אלה בן גיא</v>
+        <v>עדן בחרוף</v>
       </c>
       <c r="B42" t="str">
-        <v>401</v>
+        <v>user.413.31@laundry.app</v>
       </c>
       <c r="C42" t="str">
-        <v>user.401.41@laundry.app</v>
-      </c>
-      <c r="D42" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D42">
+        <v>16</v>
+      </c>
+      <c r="E42" t="str">
+        <v>413</v>
+      </c>
+      <c r="F42" t="str">
+        <v>0548754057</v>
+      </c>
+      <c r="G42" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>שיר סוויסה</v>
+        <v>עידן חן סימנטוב</v>
       </c>
       <c r="B43" t="str">
-        <v>401</v>
+        <v>user.217.25@laundry.app</v>
       </c>
       <c r="C43" t="str">
-        <v>user.401.42@laundry.app</v>
-      </c>
-      <c r="D43" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D43">
+        <v>16</v>
+      </c>
+      <c r="E43" t="str">
+        <v>217</v>
+      </c>
+      <c r="F43" t="str">
+        <v>0525458493</v>
+      </c>
+      <c r="G43" t="str">
+        <v>מנהל</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>עמית שושנה</v>
+        <v>עילי גולדשטיין</v>
       </c>
       <c r="B44" t="str">
-        <v>405</v>
+        <v>user.219.5@laundry.app</v>
       </c>
       <c r="C44" t="str">
-        <v>user.405.43@laundry.app</v>
-      </c>
-      <c r="D44" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D44">
+        <v>16</v>
+      </c>
+      <c r="E44" t="str">
+        <v>219</v>
+      </c>
+      <c r="F44" t="str">
+        <v>0506502772</v>
+      </c>
+      <c r="G44" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>רוני קרפט</v>
+        <v>רוני מאירסון</v>
       </c>
       <c r="B45" t="str">
+        <v>user.405.47@laundry.app</v>
+      </c>
+      <c r="C45" t="str">
+        <v>123456</v>
+      </c>
+      <c r="D45">
+        <v>16</v>
+      </c>
+      <c r="E45" t="str">
         <v>405</v>
       </c>
-      <c r="C45" t="str">
-        <v>user.405.44@laundry.app</v>
-      </c>
-      <c r="D45" t="str">
-        <v>123456</v>
+      <c r="F45" t="str">
+        <v>0548323585</v>
+      </c>
+      <c r="G45" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>מאי אילארי</v>
+        <v>תמר נגר</v>
       </c>
       <c r="B46" t="str">
-        <v>405</v>
+        <v>user.407.55@laundry.app</v>
       </c>
       <c r="C46" t="str">
-        <v>user.405.45@laundry.app</v>
-      </c>
-      <c r="D46" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D46">
+        <v>16</v>
+      </c>
+      <c r="E46" t="str">
+        <v>407</v>
+      </c>
+      <c r="F46" t="str">
+        <v>0535215616</v>
+      </c>
+      <c r="G46" t="str">
+        <v>קצינת אימונים</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>הודיה יעקובי</v>
+        <v>אוהד אבדי</v>
       </c>
       <c r="B47" t="str">
-        <v>405</v>
+        <v>user.305.36@laundry.app</v>
       </c>
       <c r="C47" t="str">
-        <v>user.405.46@laundry.app</v>
-      </c>
-      <c r="D47" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D47">
+        <v>17</v>
+      </c>
+      <c r="E47" t="str">
+        <v>305</v>
+      </c>
+      <c r="F47" t="str">
+        <v>0558824527</v>
+      </c>
+      <c r="G47" t="str">
+        <v>סמ"פ</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>רוני מאריסון</v>
+        <v>אלון זלנפרוינד</v>
       </c>
       <c r="B48" t="str">
-        <v>405</v>
+        <v>user.307.16@laundry.app</v>
       </c>
       <c r="C48" t="str">
-        <v>user.405.47@laundry.app</v>
-      </c>
-      <c r="D48" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D48">
+        <v>17</v>
+      </c>
+      <c r="E48" t="str">
+        <v>307</v>
+      </c>
+      <c r="F48" t="str">
+        <v>0533406328</v>
+      </c>
+      <c r="G48" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ליאורה אייזק</v>
+        <v>דור מנשה קיפגן</v>
       </c>
       <c r="B49" t="str">
-        <v>405</v>
+        <v>user.217.23@laundry.app</v>
       </c>
       <c r="C49" t="str">
-        <v>user.405.48@laundry.app</v>
-      </c>
-      <c r="D49" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D49">
+        <v>17</v>
+      </c>
+      <c r="E49" t="str">
+        <v>217</v>
+      </c>
+      <c r="F49" t="str">
+        <v>0586748688</v>
+      </c>
+      <c r="G49" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>דנה פרידמן</v>
+        <v>הגרה שווגר</v>
       </c>
       <c r="B50" t="str">
+        <v>user.409.50@laundry.app</v>
+      </c>
+      <c r="C50" t="str">
+        <v>123456</v>
+      </c>
+      <c r="D50">
+        <v>17</v>
+      </c>
+      <c r="E50" t="str">
         <v>409</v>
       </c>
-      <c r="C50" t="str">
-        <v>user.409.49@laundry.app</v>
-      </c>
-      <c r="D50" t="str">
-        <v>123456</v>
+      <c r="F50" t="str">
+        <v>0535315557</v>
+      </c>
+      <c r="G50" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>הגרה שווגר</v>
+        <v>טל הנגבי</v>
       </c>
       <c r="B51" t="str">
-        <v>409</v>
+        <v>user.403.7@laundry.app</v>
       </c>
       <c r="C51" t="str">
-        <v>user.409.50@laundry.app</v>
-      </c>
-      <c r="D51" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D51">
+        <v>17</v>
+      </c>
+      <c r="E51" t="str">
+        <v>403</v>
+      </c>
+      <c r="F51" t="str">
+        <v>0552250525</v>
+      </c>
+      <c r="G51" t="str">
+        <v>קצינת מבצעים פלוגתית</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>רעות ניר</v>
+        <v>יהונתן אבוקרט</v>
       </c>
       <c r="B52" t="str">
-        <v>409</v>
+        <v>user.219.3@laundry.app</v>
       </c>
       <c r="C52" t="str">
-        <v>user.409.51@laundry.app</v>
-      </c>
-      <c r="D52" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D52">
+        <v>17</v>
+      </c>
+      <c r="E52" t="str">
+        <v>219</v>
+      </c>
+      <c r="F52" t="str">
+        <v>0543836063</v>
+      </c>
+      <c r="G52" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>נגה ברק</v>
+        <v>יובל ישר</v>
       </c>
       <c r="B53" t="str">
-        <v>409</v>
+        <v>user.219.2@laundry.app</v>
       </c>
       <c r="C53" t="str">
-        <v>user.409.52@laundry.app</v>
-      </c>
-      <c r="D53" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D53">
+        <v>17</v>
+      </c>
+      <c r="E53" t="str">
+        <v>219</v>
+      </c>
+      <c r="F53" t="str">
+        <v>0584985058</v>
+      </c>
+      <c r="G53" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>נטע וילונסקי</v>
+        <v>ליאורה אייזק</v>
       </c>
       <c r="B54" t="str">
-        <v>409</v>
+        <v>user.405.48@laundry.app</v>
       </c>
       <c r="C54" t="str">
-        <v>user.409.53@laundry.app</v>
-      </c>
-      <c r="D54" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D54">
+        <v>17</v>
+      </c>
+      <c r="E54" t="str">
+        <v>405</v>
+      </c>
+      <c r="F54" t="str">
+        <v>0584143838</v>
+      </c>
+      <c r="G54" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>עמנואל נמרודי</v>
+        <v>נגה ברק</v>
       </c>
       <c r="B55" t="str">
+        <v>user.409.52@laundry.app</v>
+      </c>
+      <c r="C55" t="str">
+        <v>123456</v>
+      </c>
+      <c r="D55">
+        <v>17</v>
+      </c>
+      <c r="E55" t="str">
         <v>409</v>
       </c>
-      <c r="C55" t="str">
-        <v>user.409.54@laundry.app</v>
-      </c>
-      <c r="D55" t="str">
-        <v>123456</v>
+      <c r="F55" t="str">
+        <v>0535050505</v>
+      </c>
+      <c r="G55" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>תמר נגר</v>
+        <v>נעם שילה</v>
       </c>
       <c r="B56" t="str">
+        <v>user.407.60@laundry.app</v>
+      </c>
+      <c r="C56" t="str">
+        <v>123456</v>
+      </c>
+      <c r="D56">
+        <v>17</v>
+      </c>
+      <c r="E56" t="str">
         <v>407</v>
       </c>
-      <c r="C56" t="str">
-        <v>user.407.55@laundry.app</v>
-      </c>
-      <c r="D56" t="str">
-        <v>123456</v>
+      <c r="F56" t="str">
+        <v>0526631405</v>
+      </c>
+      <c r="G56" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ליה אלון</v>
+        <v>עדי ויינשטיין</v>
       </c>
       <c r="B57" t="str">
-        <v>407</v>
+        <v>user.307.15@laundry.app</v>
       </c>
       <c r="C57" t="str">
-        <v>user.407.56@laundry.app</v>
-      </c>
-      <c r="D57" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D57">
+        <v>17</v>
+      </c>
+      <c r="E57" t="str">
+        <v>307</v>
+      </c>
+      <c r="F57" t="str">
+        <v>0542225007</v>
+      </c>
+      <c r="G57" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>טליה פרסט</v>
+        <v>עידן טורקיה</v>
       </c>
       <c r="B58" t="str">
-        <v>407</v>
+        <v>user.305.34@laundry.app</v>
       </c>
       <c r="C58" t="str">
-        <v>user.407.57@laundry.app</v>
-      </c>
-      <c r="D58" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D58">
+        <v>17</v>
+      </c>
+      <c r="E58" t="str">
+        <v>305</v>
+      </c>
+      <c r="F58" t="str">
+        <v>0503376225</v>
+      </c>
+      <c r="G58" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>נעמה לוי</v>
+        <v>עמנואל נמרודי</v>
       </c>
       <c r="B59" t="str">
-        <v>407</v>
+        <v>user.409.54@laundry.app</v>
       </c>
       <c r="C59" t="str">
-        <v>user.407.58@laundry.app</v>
-      </c>
-      <c r="D59" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D59">
+        <v>17</v>
+      </c>
+      <c r="E59" t="str">
+        <v>409</v>
+      </c>
+      <c r="F59" t="str">
+        <v>0549577777</v>
+      </c>
+      <c r="G59" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>שילת נוימן</v>
+        <v>רועי דדון</v>
       </c>
       <c r="B60" t="str">
-        <v>407</v>
+        <v>user.219.1@laundry.app</v>
       </c>
       <c r="C60" t="str">
-        <v>user.407.59@laundry.app</v>
-      </c>
-      <c r="D60" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D60">
+        <v>17</v>
+      </c>
+      <c r="E60" t="str">
+        <v>219</v>
+      </c>
+      <c r="F60" t="str">
+        <v>0525988918</v>
+      </c>
+      <c r="G60" t="str">
+        <v>חייל</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>נעם שילה</v>
+        <v>רננה ישראלוב</v>
       </c>
       <c r="B61" t="str">
-        <v>407</v>
+        <v>user.411.20@laundry.app</v>
       </c>
       <c r="C61" t="str">
-        <v>user.407.60@laundry.app</v>
-      </c>
-      <c r="D61" t="str">
-        <v>123456</v>
+        <v>123456</v>
+      </c>
+      <c r="D61">
+        <v>17</v>
+      </c>
+      <c r="E61" t="str">
+        <v>411</v>
+      </c>
+      <c r="F61" t="str">
+        <v>0502859111</v>
+      </c>
+      <c r="G61" t="str">
+        <v>חייל</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G61"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update user logins: civilian emails + personal ID as password
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/users-login-list.xlsx
+++ b/users-login-list.xlsx
@@ -416,7 +416,7 @@
         <v>אימייל (שם משתמש)</v>
       </c>
       <c r="C1" t="str">
-        <v>סיסמה</v>
+        <v>סיסמה (מספר אישי)</v>
       </c>
       <c r="D1" t="str">
         <v>צוות</v>
@@ -436,10 +436,10 @@
         <v>אייל מוזר</v>
       </c>
       <c r="B2" t="str">
-        <v>user.217.24@laundry.app</v>
+        <v>mozer.eyal@gmail.com</v>
       </c>
       <c r="C2" t="str">
-        <v>123456</v>
+        <v>9338360</v>
       </c>
       <c r="D2">
         <v>14</v>
@@ -459,10 +459,10 @@
         <v>אלה בן גיא</v>
       </c>
       <c r="B3" t="str">
-        <v>user.401.41@laundry.app</v>
+        <v>ellabenguy2225@gmail.com</v>
       </c>
       <c r="C3" t="str">
-        <v>123456</v>
+        <v>9327853</v>
       </c>
       <c r="D3">
         <v>14</v>
@@ -482,10 +482,10 @@
         <v>דולב כהן</v>
       </c>
       <c r="B4" t="str">
-        <v>user.219.6@laundry.app</v>
+        <v>sukcfvi13@gmail.com</v>
       </c>
       <c r="C4" t="str">
-        <v>123456</v>
+        <v>9227516</v>
       </c>
       <c r="D4">
         <v>14</v>
@@ -508,7 +508,7 @@
         <v>user.401.39@laundry.app</v>
       </c>
       <c r="C5" t="str">
-        <v>123456</v>
+        <v>dotan2026</v>
       </c>
       <c r="D5">
         <v>14</v>
@@ -525,10 +525,10 @@
         <v>יזן כנעאן</v>
       </c>
       <c r="B6" t="str">
-        <v>user.307.14@laundry.app</v>
+        <v>yazankenaan@gmail.com</v>
       </c>
       <c r="C6" t="str">
-        <v>123456</v>
+        <v>9570550</v>
       </c>
       <c r="D6">
         <v>14</v>
@@ -551,7 +551,7 @@
         <v>user.401.40@laundry.app</v>
       </c>
       <c r="C7" t="str">
-        <v>123456</v>
+        <v>dotan2026</v>
       </c>
       <c r="D7">
         <v>14</v>
@@ -568,10 +568,10 @@
         <v>כפיר ברמן</v>
       </c>
       <c r="B8" t="str">
-        <v>user.305.32@laundry.app</v>
+        <v>kfir2727@gmail.com</v>
       </c>
       <c r="C8" t="str">
-        <v>123456</v>
+        <v>9277951</v>
       </c>
       <c r="D8">
         <v>14</v>
@@ -591,10 +591,10 @@
         <v>כרמל מורן</v>
       </c>
       <c r="B9" t="str">
-        <v>user.401.38@laundry.app</v>
+        <v>carmel6530@gmail.com</v>
       </c>
       <c r="C9" t="str">
-        <v>123456</v>
+        <v>9330305</v>
       </c>
       <c r="D9">
         <v>14</v>
@@ -614,10 +614,10 @@
         <v>לייה אלון</v>
       </c>
       <c r="B10" t="str">
-        <v>user.407.56@laundry.app</v>
+        <v>liya20061144@gmail.com</v>
       </c>
       <c r="C10" t="str">
-        <v>123456</v>
+        <v>9619397</v>
       </c>
       <c r="D10">
         <v>14</v>
@@ -637,10 +637,10 @@
         <v>מאי צימרמן</v>
       </c>
       <c r="B11" t="str">
-        <v>user.403.8@laundry.app</v>
+        <v>mayzimer1974@gmail.com</v>
       </c>
       <c r="C11" t="str">
-        <v>123456</v>
+        <v>9469530</v>
       </c>
       <c r="D11">
         <v>14</v>
@@ -660,10 +660,10 @@
         <v>ענבר שלח</v>
       </c>
       <c r="B12" t="str">
-        <v>user.411.21@laundry.app</v>
+        <v>inbar879@gmail.com</v>
       </c>
       <c r="C12" t="str">
-        <v>123456</v>
+        <v>9391443</v>
       </c>
       <c r="D12">
         <v>14</v>
@@ -683,10 +683,10 @@
         <v>פיונה פנג</v>
       </c>
       <c r="B13" t="str">
-        <v>user.403.9@laundry.app</v>
+        <v>fionasivv@gmail.com</v>
       </c>
       <c r="C13" t="str">
-        <v>123456</v>
+        <v>9178875</v>
       </c>
       <c r="D13">
         <v>14</v>
@@ -706,10 +706,10 @@
         <v>רוני קרפט</v>
       </c>
       <c r="B14" t="str">
-        <v>user.405.44@laundry.app</v>
+        <v>kraftroni@gmail.com</v>
       </c>
       <c r="C14" t="str">
-        <v>123456</v>
+        <v>9555602</v>
       </c>
       <c r="D14">
         <v>14</v>
@@ -729,10 +729,10 @@
         <v>רותם כוכבי</v>
       </c>
       <c r="B15" t="str">
-        <v>user.413.28@laundry.app</v>
+        <v>rotemkochavi27@gmail.com</v>
       </c>
       <c r="C15" t="str">
-        <v>123456</v>
+        <v>9497453</v>
       </c>
       <c r="D15">
         <v>14</v>
@@ -752,10 +752,10 @@
         <v>רעות ניר</v>
       </c>
       <c r="B16" t="str">
-        <v>user.409.51@laundry.app</v>
+        <v>reutnir9@gmail.com</v>
       </c>
       <c r="C16" t="str">
-        <v>123456</v>
+        <v>9448464</v>
       </c>
       <c r="D16">
         <v>14</v>
@@ -775,10 +775,10 @@
         <v>אופק מזור</v>
       </c>
       <c r="B17" t="str">
-        <v>user.307.13@laundry.app</v>
+        <v>ofekmazorek@gmail.com</v>
       </c>
       <c r="C17" t="str">
-        <v>123456</v>
+        <v>9538466</v>
       </c>
       <c r="D17">
         <v>15</v>
@@ -798,10 +798,10 @@
         <v>איתן אונגר</v>
       </c>
       <c r="B18" t="str">
-        <v>user.305.33@laundry.app</v>
+        <v>erangers22@gmail.com</v>
       </c>
       <c r="C18" t="str">
-        <v>123456</v>
+        <v>9296359</v>
       </c>
       <c r="D18">
         <v>15</v>
@@ -821,10 +821,10 @@
         <v>דנה פרידמן</v>
       </c>
       <c r="B19" t="str">
-        <v>user.409.49@laundry.app</v>
+        <v>fridmandana189@gmail.com</v>
       </c>
       <c r="C19" t="str">
-        <v>123456</v>
+        <v>9529116</v>
       </c>
       <c r="D19">
         <v>15</v>
@@ -844,10 +844,10 @@
         <v>הודיה יעקבי</v>
       </c>
       <c r="B20" t="str">
-        <v>user.405.46@laundry.app</v>
+        <v>hodayayakobi@gmail.com</v>
       </c>
       <c r="C20" t="str">
-        <v>123456</v>
+        <v>9361923</v>
       </c>
       <c r="D20">
         <v>15</v>
@@ -867,10 +867,10 @@
         <v>הללי בר יוסף</v>
       </c>
       <c r="B21" t="str">
-        <v>user.401.37@laundry.app</v>
+        <v>halleliby@gmail.com</v>
       </c>
       <c r="C21" t="str">
-        <v>123456</v>
+        <v>9574392</v>
       </c>
       <c r="D21">
         <v>15</v>
@@ -890,10 +890,10 @@
         <v>ורוורה טופן</v>
       </c>
       <c r="B22" t="str">
-        <v>user.411.17@laundry.app</v>
+        <v>varvaratofa@gmail.com</v>
       </c>
       <c r="C22" t="str">
-        <v>123456</v>
+        <v>9663012</v>
       </c>
       <c r="D22">
         <v>15</v>
@@ -916,7 +916,7 @@
         <v>user.407.57@laundry.app</v>
       </c>
       <c r="C23" t="str">
-        <v>123456</v>
+        <v>dotan2026</v>
       </c>
       <c r="D23">
         <v>15</v>
@@ -933,10 +933,10 @@
         <v>יניב גופמן</v>
       </c>
       <c r="B24" t="str">
-        <v>user.217.26@laundry.app</v>
+        <v>yanivgofman@gmail.com</v>
       </c>
       <c r="C24" t="str">
-        <v>123456</v>
+        <v>9363335</v>
       </c>
       <c r="D24">
         <v>15</v>
@@ -956,10 +956,10 @@
         <v>יערה רחוביצקי</v>
       </c>
       <c r="B25" t="str">
-        <v>user.413.30@laundry.app</v>
+        <v>yaara.rej@gmail.com</v>
       </c>
       <c r="C25" t="str">
-        <v>123456</v>
+        <v>9556782</v>
       </c>
       <c r="D25">
         <v>15</v>
@@ -979,10 +979,10 @@
         <v>מאי אילארי</v>
       </c>
       <c r="B26" t="str">
-        <v>user.405.45@laundry.app</v>
+        <v>mayilary@gmail.com</v>
       </c>
       <c r="C26" t="str">
-        <v>123456</v>
+        <v>9624875</v>
       </c>
       <c r="D26">
         <v>15</v>
@@ -1002,10 +1002,10 @@
         <v>מיקה חיים</v>
       </c>
       <c r="B27" t="str">
-        <v>user.403.11@laundry.app</v>
+        <v>mikahaim12345@gmail.com</v>
       </c>
       <c r="C27" t="str">
-        <v>123456</v>
+        <v>9722790</v>
       </c>
       <c r="D27">
         <v>15</v>
@@ -1025,10 +1025,10 @@
         <v>נעמה לביא</v>
       </c>
       <c r="B28" t="str">
-        <v>user.407.58@laundry.app</v>
+        <v>naamalavi0205@gmail.com</v>
       </c>
       <c r="C28" t="str">
-        <v>123456</v>
+        <v>9619020</v>
       </c>
       <c r="D28">
         <v>15</v>
@@ -1048,10 +1048,10 @@
         <v>עילי בן אברהם</v>
       </c>
       <c r="B29" t="str">
-        <v>user.219.4@laundry.app</v>
+        <v>illayba2016@gmail.com</v>
       </c>
       <c r="C29" t="str">
-        <v>123456</v>
+        <v>9530796</v>
       </c>
       <c r="D29">
         <v>15</v>
@@ -1074,7 +1074,7 @@
         <v>user.405.43@laundry.app</v>
       </c>
       <c r="C30" t="str">
-        <v>123456</v>
+        <v>dotan2026</v>
       </c>
       <c r="D30">
         <v>15</v>
@@ -1091,10 +1091,10 @@
         <v>שילת נוימן</v>
       </c>
       <c r="B31" t="str">
-        <v>user.407.59@laundry.app</v>
+        <v>shilatnoy05@gmail.com</v>
       </c>
       <c r="C31" t="str">
-        <v>123456</v>
+        <v>9346959</v>
       </c>
       <c r="D31">
         <v>15</v>
@@ -1114,10 +1114,10 @@
         <v>שיר סויסה</v>
       </c>
       <c r="B32" t="str">
-        <v>user.401.42@laundry.app</v>
+        <v>shirswisa2005@gmail.com</v>
       </c>
       <c r="C32" t="str">
-        <v>123456</v>
+        <v>9459947</v>
       </c>
       <c r="D32">
         <v>15</v>
@@ -1137,10 +1137,10 @@
         <v>שני זידמן</v>
       </c>
       <c r="B33" t="str">
-        <v>user.411.19@laundry.app</v>
+        <v>shani.zaidman.2006@gmail.com</v>
       </c>
       <c r="C33" t="str">
-        <v>123456</v>
+        <v>9506588</v>
       </c>
       <c r="D33">
         <v>15</v>
@@ -1160,10 +1160,10 @@
         <v>אורי חדד</v>
       </c>
       <c r="B34" t="str">
-        <v>user.305.35@laundry.app</v>
+        <v>orihadad2007@gmail.com</v>
       </c>
       <c r="C34" t="str">
-        <v>123456</v>
+        <v>9713314</v>
       </c>
       <c r="D34">
         <v>16</v>
@@ -1183,10 +1183,10 @@
         <v>אלה פלד</v>
       </c>
       <c r="B35" t="str">
-        <v>user.413.29@laundry.app</v>
+        <v>peled.e.20@gmail.com</v>
       </c>
       <c r="C35" t="str">
-        <v>123456</v>
+        <v>9419715</v>
       </c>
       <c r="D35">
         <v>16</v>
@@ -1206,10 +1206,10 @@
         <v>הילה פינצי</v>
       </c>
       <c r="B36" t="str">
-        <v>user.403.10@laundry.app</v>
+        <v>hillafin@gmail.com</v>
       </c>
       <c r="C36" t="str">
-        <v>123456</v>
+        <v>9652742</v>
       </c>
       <c r="D36">
         <v>16</v>
@@ -1229,10 +1229,10 @@
         <v>יהלי לוי</v>
       </c>
       <c r="B37" t="str">
-        <v>user.413.27@laundry.app</v>
+        <v>yahelilevi2005@gmail.com</v>
       </c>
       <c r="C37" t="str">
-        <v>123456</v>
+        <v>9407817</v>
       </c>
       <c r="D37">
         <v>16</v>
@@ -1252,10 +1252,10 @@
         <v>מעיין מרדכי</v>
       </c>
       <c r="B38" t="str">
-        <v>user.411.22@laundry.app</v>
+        <v>maayan04mor@gmail.com</v>
       </c>
       <c r="C38" t="str">
-        <v>123456</v>
+        <v>9193974</v>
       </c>
       <c r="D38">
         <v>16</v>
@@ -1275,10 +1275,10 @@
         <v>נועה בלפור</v>
       </c>
       <c r="B39" t="str">
-        <v>user.411.18@laundry.app</v>
+        <v>noa.balfour@gmail.com</v>
       </c>
       <c r="C39" t="str">
-        <v>123456</v>
+        <v>9390128</v>
       </c>
       <c r="D39">
         <v>16</v>
@@ -1298,10 +1298,10 @@
         <v>נועה גלמן</v>
       </c>
       <c r="B40" t="str">
-        <v>user.403.12@laundry.app</v>
+        <v>noa1.gelman@gmail.com</v>
       </c>
       <c r="C40" t="str">
-        <v>123456</v>
+        <v>9497489</v>
       </c>
       <c r="D40">
         <v>16</v>
@@ -1321,10 +1321,10 @@
         <v>נטע וילונסקי</v>
       </c>
       <c r="B41" t="str">
-        <v>user.409.53@laundry.app</v>
+        <v>nettawielunski@gmail.com</v>
       </c>
       <c r="C41" t="str">
-        <v>123456</v>
+        <v>9378176</v>
       </c>
       <c r="D41">
         <v>16</v>
@@ -1344,10 +1344,10 @@
         <v>עדן בחרוף</v>
       </c>
       <c r="B42" t="str">
-        <v>user.413.31@laundry.app</v>
+        <v>bbajaroff@gmail.com</v>
       </c>
       <c r="C42" t="str">
-        <v>123456</v>
+        <v>9221859</v>
       </c>
       <c r="D42">
         <v>16</v>
@@ -1367,10 +1367,10 @@
         <v>עידן חן סימנטוב</v>
       </c>
       <c r="B43" t="str">
-        <v>user.217.25@laundry.app</v>
+        <v>idan052545@gmail.com</v>
       </c>
       <c r="C43" t="str">
-        <v>123456</v>
+        <v>9075187</v>
       </c>
       <c r="D43">
         <v>16</v>
@@ -1390,10 +1390,10 @@
         <v>עילי גולדשטיין</v>
       </c>
       <c r="B44" t="str">
-        <v>user.219.5@laundry.app</v>
+        <v>ilaykey@gmail.com</v>
       </c>
       <c r="C44" t="str">
-        <v>123456</v>
+        <v>9257449</v>
       </c>
       <c r="D44">
         <v>16</v>
@@ -1413,10 +1413,10 @@
         <v>רוני מאירסון</v>
       </c>
       <c r="B45" t="str">
-        <v>user.405.47@laundry.app</v>
+        <v>roni.meirson@gmail.com</v>
       </c>
       <c r="C45" t="str">
-        <v>123456</v>
+        <v>9413145</v>
       </c>
       <c r="D45">
         <v>16</v>
@@ -1436,10 +1436,10 @@
         <v>תמר נגר</v>
       </c>
       <c r="B46" t="str">
-        <v>user.407.55@laundry.app</v>
+        <v>tamarnagar27@gmail.com</v>
       </c>
       <c r="C46" t="str">
-        <v>123456</v>
+        <v>9421803</v>
       </c>
       <c r="D46">
         <v>16</v>
@@ -1459,10 +1459,10 @@
         <v>אוהד אבדי</v>
       </c>
       <c r="B47" t="str">
-        <v>user.305.36@laundry.app</v>
+        <v>ohad9623@gmail.com</v>
       </c>
       <c r="C47" t="str">
-        <v>123456</v>
+        <v>9351505</v>
       </c>
       <c r="D47">
         <v>17</v>
@@ -1482,10 +1482,10 @@
         <v>אלון זלנפרוינד</v>
       </c>
       <c r="B48" t="str">
-        <v>user.307.16@laundry.app</v>
+        <v>alonseel@gmail.com</v>
       </c>
       <c r="C48" t="str">
-        <v>123456</v>
+        <v>9219963</v>
       </c>
       <c r="D48">
         <v>17</v>
@@ -1505,10 +1505,10 @@
         <v>דור מנשה קיפגן</v>
       </c>
       <c r="B49" t="str">
-        <v>user.217.23@laundry.app</v>
+        <v>dorm732@gmail.com</v>
       </c>
       <c r="C49" t="str">
-        <v>123456</v>
+        <v>8507348</v>
       </c>
       <c r="D49">
         <v>17</v>
@@ -1528,10 +1528,10 @@
         <v>הגרה שווגר</v>
       </c>
       <c r="B50" t="str">
-        <v>user.409.50@laundry.app</v>
+        <v>hagara.schwager@gmail.com</v>
       </c>
       <c r="C50" t="str">
-        <v>123456</v>
+        <v>9180598</v>
       </c>
       <c r="D50">
         <v>17</v>
@@ -1551,10 +1551,10 @@
         <v>טל הנגבי</v>
       </c>
       <c r="B51" t="str">
-        <v>user.403.7@laundry.app</v>
+        <v>talushhanegbi@gmail.com</v>
       </c>
       <c r="C51" t="str">
-        <v>123456</v>
+        <v>9379869</v>
       </c>
       <c r="D51">
         <v>17</v>
@@ -1574,10 +1574,10 @@
         <v>יהונתן אבוקרט</v>
       </c>
       <c r="B52" t="str">
-        <v>user.219.3@laundry.app</v>
+        <v>yhonatan5913@gmail.com</v>
       </c>
       <c r="C52" t="str">
-        <v>123456</v>
+        <v>9433520</v>
       </c>
       <c r="D52">
         <v>17</v>
@@ -1597,10 +1597,10 @@
         <v>יובל ישר</v>
       </c>
       <c r="B53" t="str">
-        <v>user.219.2@laundry.app</v>
+        <v>yasharyuval10@gmail.com</v>
       </c>
       <c r="C53" t="str">
-        <v>123456</v>
+        <v>9692159</v>
       </c>
       <c r="D53">
         <v>17</v>
@@ -1620,10 +1620,10 @@
         <v>ליאורה אייזק</v>
       </c>
       <c r="B54" t="str">
-        <v>user.405.48@laundry.app</v>
+        <v>lioraizsak@gmail.com</v>
       </c>
       <c r="C54" t="str">
-        <v>123456</v>
+        <v>9451890</v>
       </c>
       <c r="D54">
         <v>17</v>
@@ -1643,10 +1643,10 @@
         <v>נגה ברק</v>
       </c>
       <c r="B55" t="str">
-        <v>user.409.52@laundry.app</v>
+        <v>nogabarak2@gmail.com</v>
       </c>
       <c r="C55" t="str">
-        <v>123456</v>
+        <v>9530304</v>
       </c>
       <c r="D55">
         <v>17</v>
@@ -1666,10 +1666,10 @@
         <v>נעם שילה</v>
       </c>
       <c r="B56" t="str">
-        <v>user.407.60@laundry.app</v>
+        <v>noamshilo10@gmail.com</v>
       </c>
       <c r="C56" t="str">
-        <v>123456</v>
+        <v>9345422</v>
       </c>
       <c r="D56">
         <v>17</v>
@@ -1689,10 +1689,10 @@
         <v>עדי ויינשטיין</v>
       </c>
       <c r="B57" t="str">
-        <v>user.307.15@laundry.app</v>
+        <v>adi92005@gmail.com</v>
       </c>
       <c r="C57" t="str">
-        <v>123456</v>
+        <v>9336308</v>
       </c>
       <c r="D57">
         <v>17</v>
@@ -1712,10 +1712,10 @@
         <v>עידן טורקיה</v>
       </c>
       <c r="B58" t="str">
-        <v>user.305.34@laundry.app</v>
+        <v>idant95@gmail.com</v>
       </c>
       <c r="C58" t="str">
-        <v>123456</v>
+        <v>9423591</v>
       </c>
       <c r="D58">
         <v>17</v>
@@ -1735,10 +1735,10 @@
         <v>עמנואל נמרודי</v>
       </c>
       <c r="B59" t="str">
-        <v>user.409.54@laundry.app</v>
+        <v>emnimrodi@gmail.com</v>
       </c>
       <c r="C59" t="str">
-        <v>123456</v>
+        <v>9391594</v>
       </c>
       <c r="D59">
         <v>17</v>
@@ -1758,10 +1758,10 @@
         <v>רועי דדון</v>
       </c>
       <c r="B60" t="str">
-        <v>user.219.1@laundry.app</v>
+        <v>roidadon991@gmail.com</v>
       </c>
       <c r="C60" t="str">
-        <v>123456</v>
+        <v>9395097</v>
       </c>
       <c r="D60">
         <v>17</v>
@@ -1781,10 +1781,10 @@
         <v>רננה ישראלוב</v>
       </c>
       <c r="B61" t="str">
-        <v>user.411.20@laundry.app</v>
+        <v>israelovrenana@gmail.com</v>
       </c>
       <c r="C61" t="str">
-        <v>123456</v>
+        <v>9369390</v>
       </c>
       <c r="D61">
         <v>17</v>

</xml_diff>